<commit_message>
feat: add Page 2 (Slide 2: Skema Kerjasama & Bagi Hasil) and update master Excel Sheet 07
</commit_message>
<xml_diff>
--- a/dashboard PCO/Simulasi_Investasi_dan_Produksi_PCO.xlsx
+++ b/dashboard PCO/Simulasi_Investasi_dan_Produksi_PCO.xlsx
@@ -13,6 +13,7 @@
     <sheet name="04_Data_Asal_Aset_Depresiasi" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="05_Data_Asal_Penjualan_Invoice" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="06_Pengolahan_Laba_Rugi" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="07_Skema_Kerjasama_Bagi_Hasil" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,19 +22,22 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="13">
     <numFmt numFmtId="164" formatCode="&quot;Rp&quot;#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot; Ton/hari (30.000 kg)&quot;"/>
     <numFmt numFmtId="166" formatCode="#,##0&quot; Ton/hari (20.000 kg)&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0&quot; jam&quot;"/>
     <numFmt numFmtId="168" formatCode="#,##0&quot; hari&quot;"/>
-    <numFmt numFmtId="169" formatCode="#,##0&quot; kg (± 520,00 ton)&quot;"/>
-    <numFmt numFmtId="170" formatCode="&quot;Rp&quot;#,##0&quot;/kg&quot;"/>
+    <numFmt numFmtId="169" formatCode="&quot;Rp&quot;#,##0&quot;/kg&quot;"/>
+    <numFmt numFmtId="170" formatCode="#,##0&quot; kg (± 520,00 ton)&quot;"/>
     <numFmt numFmtId="171" formatCode="#,##0&quot; Ton/hari&quot;"/>
     <numFmt numFmtId="172" formatCode="#,##0&quot; kg&quot;"/>
     <numFmt numFmtId="173" formatCode="#,##0&quot; Ton&quot;"/>
+    <numFmt numFmtId="174" formatCode="Rp #,##0"/>
+    <numFmt numFmtId="175" formatCode="0.00 Bulan"/>
+    <numFmt numFmtId="176" formatCode="0.00 Tahun"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="40">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -192,8 +196,75 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000C2B53"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000C2B53"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000C2B53"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <i val="1"/>
+      <color rgb="00475569"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="0064748B"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001E40AF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -308,8 +379,20 @@
         <bgColor rgb="001E293B"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000C2B53"/>
+        <bgColor rgb="000C2B53"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000A6358"/>
+        <bgColor rgb="000A6358"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="64">
+  <borders count="118">
     <border>
       <left/>
       <right/>
@@ -1199,11 +1282,613 @@
         <color rgb="001E293B"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F766E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000F766E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="000F766E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000F766E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="000F766E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00065F46"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00065F46"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00065F46"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00334155"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00334155"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001E3A8A"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00334155"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="00334155"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00334155"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="00334155"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000369A1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="000369A1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="000369A1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="000369A1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F766E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F766E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00065F46"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="00065F46"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00065F46"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="00065F46"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001E3A8A"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="001E3A8A"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001E3A8A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="001E3A8A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00D97706"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00D97706"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000369A1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00D97706"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="00D97706"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00D97706"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="00D97706"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00047857"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="00047857"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00047857"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="medium">
+        <color rgb="00047857"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="double">
+        <color rgb="000F172A"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="236">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1295,7 +1980,7 @@
     <xf numFmtId="168" fontId="5" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1306,7 +1991,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="8" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="170" fontId="8" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="16" borderId="45" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1314,7 +1999,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="46" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1327,7 +2012,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="13" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1461,7 +2146,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="8" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="8" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="8" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1489,6 +2174,147 @@
     <xf numFmtId="10" fontId="6" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="100" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="101" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="111" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="112" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="97" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="75" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="82" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="85" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="8" fillId="7" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="80" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="81" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="104" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="107" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="108" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="102" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="103" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="8" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="31" fillId="21" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="32" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="13" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="32" fillId="13" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="32" fillId="5" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="5" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="33" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="32" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="11" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="11" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="37" fillId="0" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="114" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="114" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="114" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="19" fillId="13" borderId="114" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="11" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="39" fillId="5" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="36" fillId="11" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="19" fillId="13" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="114" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="114" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="11" borderId="114" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="36" fillId="11" borderId="114" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="117" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="174" fontId="36" fillId="0" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="175" fontId="19" fillId="13" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="19" fillId="13" borderId="113" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="113" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1884,29 +2710,28 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>1. INVESTASI</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="5" t="n"/>
+      <c r="B4" s="147" t="n"/>
+      <c r="C4" s="148" t="n"/>
       <c r="E4" s="6" t="inlineStr">
         <is>
           <t>4. STRUKTUR HPP</t>
         </is>
       </c>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
+      <c r="F4" s="149" t="n"/>
+      <c r="G4" s="150" t="n"/>
       <c r="I4" s="9" t="inlineStr">
         <is>
           <t>KEY HIGHLIGHTS</t>
         </is>
       </c>
-      <c r="J4" s="10" t="n"/>
-      <c r="K4" s="11" t="n"/>
+      <c r="J4" s="151" t="n"/>
+      <c r="K4" s="152" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -1914,7 +2739,7 @@
           <t>4 Unit Mesin (@ Rp 900 juta)</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n"/>
+      <c r="B5" s="153" t="n"/>
       <c r="C5" s="14">
         <f>04_Data_Asal_Aset_Depresiasi!E9</f>
         <v/>
@@ -1945,7 +2770,7 @@
 Investasi Rp 3,6 Miliar</t>
         </is>
       </c>
-      <c r="K5" s="20" t="n"/>
+      <c r="K5" s="154" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -1953,7 +2778,7 @@
           <t>Pembangunan Gudang</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n"/>
+      <c r="B6" s="153" t="n"/>
       <c r="C6" s="14">
         <f>04_Data_Asal_Aset_Depresiasi!E10</f>
         <v/>
@@ -1972,9 +2797,9 @@
           <t>Penyesuaian CPO (Rp 2.000/kg)</t>
         </is>
       </c>
-      <c r="I6" s="24" t="n"/>
-      <c r="J6" s="13" t="n"/>
-      <c r="K6" s="20" t="n"/>
+      <c r="I6" s="155" t="n"/>
+      <c r="J6" s="156" t="n"/>
+      <c r="K6" s="157" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="25" t="inlineStr">
@@ -1982,7 +2807,7 @@
           <t>Total Investasi</t>
         </is>
       </c>
-      <c r="B7" s="26" t="n"/>
+      <c r="B7" s="158" t="n"/>
       <c r="C7" s="27">
         <f>C5+C6</f>
         <v/>
@@ -2012,7 +2837,7 @@
 Produksi Jadi (20 Ton/hari)</t>
         </is>
       </c>
-      <c r="K7" s="20" t="n"/>
+      <c r="K7" s="154" t="n"/>
     </row>
     <row r="8">
       <c r="E8" s="21" t="inlineStr">
@@ -2029,9 +2854,9 @@
           <t>Alokasi biaya gudang</t>
         </is>
       </c>
-      <c r="I8" s="24" t="n"/>
-      <c r="J8" s="13" t="n"/>
-      <c r="K8" s="20" t="n"/>
+      <c r="I8" s="155" t="n"/>
+      <c r="J8" s="156" t="n"/>
+      <c r="K8" s="157" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
@@ -2039,8 +2864,8 @@
           <t>2. KAPASITAS &amp; PRODUKSI</t>
         </is>
       </c>
-      <c r="B9" s="30" t="n"/>
-      <c r="C9" s="31" t="n"/>
+      <c r="B9" s="159" t="n"/>
+      <c r="C9" s="160" t="n"/>
       <c r="E9" s="32" t="inlineStr">
         <is>
           <t>Cash HPP</t>
@@ -2066,7 +2891,7 @@
 (520.000 kg x Rp8.300)</t>
         </is>
       </c>
-      <c r="K9" s="20" t="n"/>
+      <c r="K9" s="154" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="36" t="inlineStr">
@@ -2074,7 +2899,7 @@
           <t>Kapasitas sebelum yield</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n"/>
+      <c r="B10" s="153" t="n"/>
       <c r="C10" s="37">
         <f>02_Data_Asal_Produksi_Harian!M4</f>
         <v/>
@@ -2093,9 +2918,9 @@
           <t>Capex Rp 5 M (5 tahun)</t>
         </is>
       </c>
-      <c r="I10" s="24" t="n"/>
-      <c r="J10" s="13" t="n"/>
-      <c r="K10" s="20" t="n"/>
+      <c r="I10" s="155" t="n"/>
+      <c r="J10" s="156" t="n"/>
+      <c r="K10" s="157" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="36" t="inlineStr">
@@ -2103,7 +2928,7 @@
           <t>Yield produksi</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n"/>
+      <c r="B11" s="153" t="n"/>
       <c r="C11" s="38">
         <f>02_Data_Asal_Produksi_Harian!M5</f>
         <v/>
@@ -2133,7 +2958,7 @@
 (Rp22,79 Miliar / tahun)</t>
         </is>
       </c>
-      <c r="K11" s="20" t="n"/>
+      <c r="K11" s="154" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="36" t="inlineStr">
@@ -2141,14 +2966,14 @@
           <t>Produk jadi setelah yield</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n"/>
+      <c r="B12" s="153" t="n"/>
       <c r="C12" s="43">
         <f>02_Data_Asal_Produksi_Harian!M6</f>
         <v/>
       </c>
-      <c r="I12" s="44" t="n"/>
-      <c r="J12" s="45" t="n"/>
-      <c r="K12" s="46" t="n"/>
+      <c r="I12" s="155" t="n"/>
+      <c r="J12" s="156" t="n"/>
+      <c r="K12" s="157" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="36" t="inlineStr">
@@ -2156,7 +2981,7 @@
           <t>Jam operasi per hari</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n"/>
+      <c r="B13" s="153" t="n"/>
       <c r="C13" s="47">
         <f>02_Data_Asal_Produksi_Harian!M7</f>
         <v/>
@@ -2166,8 +2991,8 @@
           <t>5. PROFITABILITAS</t>
         </is>
       </c>
-      <c r="F13" s="30" t="n"/>
-      <c r="G13" s="31" t="n"/>
+      <c r="F13" s="159" t="n"/>
+      <c r="G13" s="160" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="36" t="inlineStr">
@@ -2175,7 +3000,7 @@
           <t>Hari kerja per bulan</t>
         </is>
       </c>
-      <c r="B14" s="13" t="n"/>
+      <c r="B14" s="153" t="n"/>
       <c r="C14" s="48">
         <f>02_Data_Asal_Produksi_Harian!M8</f>
         <v/>
@@ -2185,18 +3010,18 @@
           <t>Harga jual</t>
         </is>
       </c>
-      <c r="F14" s="49">
+      <c r="F14" s="161">
         <f>C18</f>
         <v/>
       </c>
-      <c r="G14" s="50" t="n"/>
+      <c r="G14" s="153" t="n"/>
       <c r="I14" s="51" t="inlineStr">
         <is>
           <t>ALUR NILAI</t>
         </is>
       </c>
-      <c r="J14" s="52" t="n"/>
-      <c r="K14" s="53" t="n"/>
+      <c r="J14" s="162" t="n"/>
+      <c r="K14" s="163" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="54" t="inlineStr">
@@ -2204,8 +3029,8 @@
           <t>Produksi per bulan</t>
         </is>
       </c>
-      <c r="B15" s="55" t="n"/>
-      <c r="C15" s="56">
+      <c r="B15" s="164" t="n"/>
+      <c r="C15" s="165">
         <f>C12*C14*1000</f>
         <v/>
       </c>
@@ -2214,18 +3039,18 @@
           <t>Full HPP</t>
         </is>
       </c>
-      <c r="F15" s="49">
+      <c r="F15" s="161">
         <f>F11</f>
         <v/>
       </c>
-      <c r="G15" s="50" t="n"/>
+      <c r="G15" s="153" t="n"/>
       <c r="I15" s="57" t="inlineStr">
         <is>
           <t>Bahan Baku      ──▶  Input Curah 30 Ton/hari</t>
         </is>
       </c>
-      <c r="J15" s="13" t="n"/>
-      <c r="K15" s="58" t="n"/>
+      <c r="J15" s="166" t="n"/>
+      <c r="K15" s="153" t="n"/>
     </row>
     <row r="16">
       <c r="E16" s="59" t="inlineStr">
@@ -2233,18 +3058,18 @@
           <t>Laba per kg</t>
         </is>
       </c>
-      <c r="F16" s="60">
+      <c r="F16" s="167">
         <f>F14-F15</f>
         <v/>
       </c>
-      <c r="G16" s="50" t="n"/>
+      <c r="G16" s="153" t="n"/>
       <c r="I16" s="57" t="inlineStr">
         <is>
           <t>Proses Produksi ──▶  Pengolahan 4 Mesin (Yield 70%)</t>
         </is>
       </c>
-      <c r="J16" s="13" t="n"/>
-      <c r="K16" s="58" t="n"/>
+      <c r="J16" s="166" t="n"/>
+      <c r="K16" s="153" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="61" t="inlineStr">
@@ -2252,8 +3077,8 @@
           <t>3. HARGA JUAL &amp; OMZET</t>
         </is>
       </c>
-      <c r="B17" s="62" t="n"/>
-      <c r="C17" s="63" t="n"/>
+      <c r="B17" s="168" t="n"/>
+      <c r="C17" s="169" t="n"/>
       <c r="E17" s="64" t="inlineStr">
         <is>
           <t>Laba per bulan (520.000 kg)</t>
@@ -2263,14 +3088,14 @@
         <f>F16*C15</f>
         <v/>
       </c>
-      <c r="G17" s="50" t="n"/>
+      <c r="G17" s="153" t="n"/>
       <c r="I17" s="57" t="inlineStr">
         <is>
           <t>PCO Produk Jadi ──▶  Output Bersih 20 Ton/hari (21 Jam)</t>
         </is>
       </c>
-      <c r="J17" s="13" t="n"/>
-      <c r="K17" s="58" t="n"/>
+      <c r="J17" s="166" t="n"/>
+      <c r="K17" s="153" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="66" t="inlineStr">
@@ -2278,8 +3103,8 @@
           <t>Harga jual</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n"/>
-      <c r="C18" s="67">
+      <c r="B18" s="153" t="n"/>
+      <c r="C18" s="170">
         <f>05_Data_Asal_Penjualan_Invoice!K3</f>
         <v/>
       </c>
@@ -2292,14 +3117,14 @@
         <f>F17*12</f>
         <v/>
       </c>
-      <c r="G18" s="70" t="n"/>
+      <c r="G18" s="164" t="n"/>
       <c r="I18" s="71" t="inlineStr">
         <is>
           <t>Nilai Ekonomi   ──▶  Margin Tinggi untuk Industri</t>
         </is>
       </c>
-      <c r="J18" s="72" t="n"/>
-      <c r="K18" s="73" t="n"/>
+      <c r="J18" s="171" t="n"/>
+      <c r="K18" s="172" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="74" t="inlineStr">
@@ -2307,7 +3132,7 @@
           <t>Omzet per bulan</t>
         </is>
       </c>
-      <c r="B19" s="75" t="n"/>
+      <c r="B19" s="173" t="n"/>
       <c r="C19" s="76">
         <f>C15*C18</f>
         <v/>
@@ -2319,8 +3144,8 @@
           <t>EXECUTIVE CONCLUSION</t>
         </is>
       </c>
-      <c r="J20" s="30" t="n"/>
-      <c r="K20" s="31" t="n"/>
+      <c r="J20" s="159" t="n"/>
+      <c r="K20" s="160" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="77" t="inlineStr">
@@ -2328,19 +3153,19 @@
           <t>CATATAN PENTING</t>
         </is>
       </c>
-      <c r="B21" s="78" t="n"/>
-      <c r="C21" s="78" t="n"/>
-      <c r="D21" s="78" t="n"/>
-      <c r="E21" s="78" t="n"/>
-      <c r="F21" s="78" t="n"/>
-      <c r="G21" s="79" t="n"/>
+      <c r="B21" s="174" t="n"/>
+      <c r="C21" s="174" t="n"/>
+      <c r="D21" s="174" t="n"/>
+      <c r="E21" s="174" t="n"/>
+      <c r="F21" s="174" t="n"/>
+      <c r="G21" s="175" t="n"/>
       <c r="I21" s="80" t="inlineStr">
         <is>
           <t>Investasi kapasitas 20 Ton/hari (520 Ton/bln) memiliki potensi margin luar biasa (Laba Rp 22,79 Miliar/tahun dengan Payback Period ±2,6 Bulan atas Capex Rp 5 Miliar). Validasi biaya operasional, pasar, pajak, modal kerja, dan utilitas 21 jam/hari diperlukan sebelum keputusan final.</t>
         </is>
       </c>
-      <c r="J21" s="13" t="n"/>
-      <c r="K21" s="50" t="n"/>
+      <c r="J21" s="176" t="n"/>
+      <c r="K21" s="154" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="81" t="inlineStr">
@@ -2348,15 +3173,14 @@
           <t>1. Perhitungan di atas belum dikurangi pajak penghasilan badan.</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n"/>
-      <c r="C22" s="13" t="n"/>
-      <c r="D22" s="13" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n"/>
-      <c r="G22" s="82" t="n"/>
-      <c r="I22" s="83" t="n"/>
-      <c r="J22" s="13" t="n"/>
-      <c r="K22" s="50" t="n"/>
+      <c r="B22" s="166" t="n"/>
+      <c r="C22" s="166" t="n"/>
+      <c r="D22" s="166" t="n"/>
+      <c r="E22" s="166" t="n"/>
+      <c r="F22" s="166" t="n"/>
+      <c r="G22" s="153" t="n"/>
+      <c r="I22" s="177" t="n"/>
+      <c r="K22" s="178" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="81" t="inlineStr">
@@ -2364,15 +3188,14 @@
           <t>2. Belum termasuk bunga/modal kerja untuk skala kapasitas 520 Ton/bulan.</t>
         </is>
       </c>
-      <c r="B23" s="13" t="n"/>
-      <c r="C23" s="13" t="n"/>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
-      <c r="G23" s="82" t="n"/>
-      <c r="I23" s="83" t="n"/>
-      <c r="J23" s="13" t="n"/>
-      <c r="K23" s="50" t="n"/>
+      <c r="B23" s="166" t="n"/>
+      <c r="C23" s="166" t="n"/>
+      <c r="D23" s="166" t="n"/>
+      <c r="E23" s="166" t="n"/>
+      <c r="F23" s="166" t="n"/>
+      <c r="G23" s="153" t="n"/>
+      <c r="I23" s="177" t="n"/>
+      <c r="K23" s="178" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="81" t="inlineStr">
@@ -2380,15 +3203,14 @@
           <t>3. Belum termasuk biaya lain di luar asumsi tersebut.</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="13" t="n"/>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="82" t="n"/>
-      <c r="I24" s="83" t="n"/>
-      <c r="J24" s="13" t="n"/>
-      <c r="K24" s="50" t="n"/>
+      <c r="B24" s="166" t="n"/>
+      <c r="C24" s="166" t="n"/>
+      <c r="D24" s="166" t="n"/>
+      <c r="E24" s="166" t="n"/>
+      <c r="F24" s="166" t="n"/>
+      <c r="G24" s="153" t="n"/>
+      <c r="I24" s="177" t="n"/>
+      <c r="K24" s="178" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="84" t="inlineStr">
@@ -2396,15 +3218,15 @@
           <t>4. Angka dapat berubah sesuai kondisi aktual di lapangan.</t>
         </is>
       </c>
-      <c r="B25" s="85" t="n"/>
-      <c r="C25" s="85" t="n"/>
-      <c r="D25" s="85" t="n"/>
-      <c r="E25" s="85" t="n"/>
-      <c r="F25" s="85" t="n"/>
-      <c r="G25" s="86" t="n"/>
-      <c r="I25" s="87" t="n"/>
-      <c r="J25" s="88" t="n"/>
-      <c r="K25" s="70" t="n"/>
+      <c r="B25" s="179" t="n"/>
+      <c r="C25" s="179" t="n"/>
+      <c r="D25" s="179" t="n"/>
+      <c r="E25" s="179" t="n"/>
+      <c r="F25" s="179" t="n"/>
+      <c r="G25" s="180" t="n"/>
+      <c r="I25" s="181" t="n"/>
+      <c r="J25" s="182" t="n"/>
+      <c r="K25" s="157" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="44">
@@ -3753,7 +4575,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="95" t="inlineStr">
         <is>
@@ -3827,7 +4648,6 @@
           <t>SUBTOTAL RAW MATERIAL EFEKTIF</t>
         </is>
       </c>
-      <c r="C8" s="112" t="n"/>
       <c r="D8" s="113">
         <f>D5</f>
         <v/>
@@ -3991,7 +4811,6 @@
           <t>SUBTOTAL BIAYA PRODUKSI (OPERASIONAL PROSES)</t>
         </is>
       </c>
-      <c r="C16" s="116" t="n"/>
       <c r="D16" s="117">
         <f>SUM(D10:D14)</f>
         <v/>
@@ -4101,7 +4920,6 @@
           <t>SUBTOTAL SEWA GUDANG (ALOKASI BIAYA GUDANG)</t>
         </is>
       </c>
-      <c r="C22" s="120" t="n"/>
       <c r="D22" s="121">
         <f>SUM(D18:D20)</f>
         <v/>
@@ -4126,7 +4944,6 @@
           <t>TOTAL CASH HPP (PENGELUARAN KAS RIIL)</t>
         </is>
       </c>
-      <c r="C24" s="124" t="n"/>
       <c r="D24" s="125">
         <f>D8+D16+D22</f>
         <v/>
@@ -4143,9 +4960,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B8:C8"/>
     <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B22:C22"/>
     <mergeCell ref="B16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4184,7 +5001,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="95" t="inlineStr">
         <is>
@@ -4360,8 +5176,6 @@
           <t>SUBTOTAL 4 UNIT MESIN PRODUKSI</t>
         </is>
       </c>
-      <c r="C9" s="111" t="n"/>
-      <c r="D9" s="111" t="n"/>
       <c r="E9" s="128">
         <f>SUM(E5:E8)</f>
         <v/>
@@ -4414,8 +5228,6 @@
           <t>TOTAL INVESTASI (CAPEX)</t>
         </is>
       </c>
-      <c r="C11" s="115" t="n"/>
-      <c r="D11" s="115" t="n"/>
       <c r="E11" s="130">
         <f>E9+E10</f>
         <v/>
@@ -4440,8 +5252,6 @@
           <t>BEBAN DEPRESIASI PER KG PRODUK JADI (ROUNDED)</t>
         </is>
       </c>
-      <c r="C13" s="123" t="n"/>
-      <c r="D13" s="123" t="n"/>
       <c r="E13" s="132">
         <f>ROUND(G11, 0)</f>
         <v/>
@@ -4509,11 +5319,10 @@
           <t>HARGA JUAL KONTRAK</t>
         </is>
       </c>
-      <c r="K3" s="135" t="n">
+      <c r="K3" s="183" t="n">
         <v>8300</v>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="95" t="inlineStr">
         <is>
@@ -5688,7 +6497,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="95" t="inlineStr">
         <is>
@@ -6042,4 +6850,797 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="199" t="inlineStr">
+        <is>
+          <t>SKEMA KERJASAMA &amp; BAGI HASIL INVESTASI PRODUKSI PCO (MINYAK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="200" t="inlineStr">
+        <is>
+          <t>Sinergi Modal dan Operasional untuk Nilai Berkelanjutan | Kapasitas 520 Ton/Bulan (Revisi Final)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="201" t="inlineStr">
+        <is>
+          <t>1. IDENTITAS &amp; PERAN PARA PIHAK DALAM KERJASAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="202" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C6" s="203" t="inlineStr">
+        <is>
+          <t>Pihak Mitra</t>
+        </is>
+      </c>
+      <c r="D6" s="203" t="inlineStr">
+        <is>
+          <t>Badan Usaha / Entitas</t>
+        </is>
+      </c>
+      <c r="E6" s="202" t="inlineStr">
+        <is>
+          <t>Porsi Bagi Hasil (EAT)</t>
+        </is>
+      </c>
+      <c r="F6" s="203" t="inlineStr">
+        <is>
+          <t>Peran &amp; Tanggung Jawab Utama</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="204" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="205" t="inlineStr">
+        <is>
+          <t>PIHAK PERTAMA (Pemodal)</t>
+        </is>
+      </c>
+      <c r="D7" s="205" t="inlineStr">
+        <is>
+          <t>PT Pioner Nusantara Sukses</t>
+        </is>
+      </c>
+      <c r="E7" s="206" t="inlineStr">
+        <is>
+          <t>60% EAT</t>
+        </is>
+      </c>
+      <c r="F7" s="205" t="inlineStr">
+        <is>
+          <t>Menanggung Capex Rp 5 M, pemilik 100% aset mesin &amp; bangunan, tidak terlibat operasional harian</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="204" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="205" t="inlineStr">
+        <is>
+          <t>PIHAK KEDUA (Pengelola)</t>
+        </is>
+      </c>
+      <c r="D8" s="205" t="inlineStr">
+        <is>
+          <t>PT. Randu Agung Bersaudara</t>
+        </is>
+      </c>
+      <c r="E8" s="207" t="inlineStr">
+        <is>
+          <t>40% EAT</t>
+        </is>
+      </c>
+      <c r="F8" s="205" t="inlineStr">
+        <is>
+          <t>Mengelola operasional produksi harian (21 jam), mengurus izin &amp; legalitas, menanggung operasional harian</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="208" t="inlineStr">
+        <is>
+          <t>2. NILAI INVESTASI (CAPEX PIHAK PERTAMA - SESUAI SLIDE SEBELUMNYA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="202" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C11" s="203" t="inlineStr">
+        <is>
+          <t>Komponen Investasi</t>
+        </is>
+      </c>
+      <c r="D11" s="202" t="inlineStr">
+        <is>
+          <t>Volume / Satuan</t>
+        </is>
+      </c>
+      <c r="E11" s="203" t="inlineStr">
+        <is>
+          <t>Nilai Investasi (Rp)</t>
+        </is>
+      </c>
+      <c r="F11" s="203" t="inlineStr">
+        <is>
+          <t>Keterangan Kepemilikan &amp; Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="204" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="205" t="inlineStr">
+        <is>
+          <t>4 Unit Mesin Produksi PCO</t>
+        </is>
+      </c>
+      <c r="D12" s="204" t="inlineStr">
+        <is>
+          <t>4 Unit @ Rp 900 Jt</t>
+        </is>
+      </c>
+      <c r="E12" s="209" t="n">
+        <v>3600000000</v>
+      </c>
+      <c r="F12" s="205" t="inlineStr">
+        <is>
+          <t>100% Milik Pihak Pertama (PT Pioner Nusantara Sukses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="204" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="205" t="inlineStr">
+        <is>
+          <t>Pembangunan &amp; Fasilitas Gudang</t>
+        </is>
+      </c>
+      <c r="D13" s="204" t="inlineStr">
+        <is>
+          <t>Infrastruktur Dasar</t>
+        </is>
+      </c>
+      <c r="E13" s="209" t="n">
+        <v>1400000000</v>
+      </c>
+      <c r="F13" s="205" t="inlineStr">
+        <is>
+          <t>Tangki penyimpanan, gudang penampungan &amp; fasilitas utilitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="210" t="inlineStr"/>
+      <c r="C14" s="211" t="inlineStr">
+        <is>
+          <t>TOTAL INVESTASI (CAPEX)</t>
+        </is>
+      </c>
+      <c r="D14" s="212" t="inlineStr">
+        <is>
+          <t>100% Pemodal</t>
+        </is>
+      </c>
+      <c r="E14" s="213">
+        <f>E12+E13</f>
+        <v/>
+      </c>
+      <c r="F14" s="211" t="inlineStr">
+        <is>
+          <t>Seluruh alat/mesin &amp; bangunan merupakan aset tetap sah Pihak Pertama</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="201" t="inlineStr">
+        <is>
+          <t>3. KEPEMILIKAN ASET &amp; HAK PENGGUNAAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="214" t="inlineStr">
+        <is>
+          <t>Aset Produksi</t>
+        </is>
+      </c>
+      <c r="C17" s="214" t="inlineStr">
+        <is>
+          <t>Status Kepemilikan: Pihak Pertama</t>
+        </is>
+      </c>
+      <c r="D17" s="214" t="inlineStr">
+        <is>
+          <t>Seluruh alat/mesin produksi dan fasilitas gudang merupakan milik sah Pihak Pertama (PT Pioner Nusantara Sukses).</t>
+        </is>
+      </c>
+      <c r="E17" s="214" t="inlineStr">
+        <is>
+          <t>Hak Operasional: Pihak Kedua</t>
+        </is>
+      </c>
+      <c r="F17" s="214" t="inlineStr">
+        <is>
+          <t>Pihak Kedua hanya berhak menggunakan alat sesuai perjanjian kerjasama. Tidak ada perpindahan kepemilikan aset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="208" t="inlineStr">
+        <is>
+          <t>4. ILUSTRASI KINERJA KEUANGAN BULANAN &amp; STRUKTUR PEMBAGIAN LABA</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="202" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C20" s="203" t="inlineStr">
+        <is>
+          <t>Uraian Komponen Finansial</t>
+        </is>
+      </c>
+      <c r="D20" s="202" t="inlineStr">
+        <is>
+          <t>Volume / Satuan Harga</t>
+        </is>
+      </c>
+      <c r="E20" s="203" t="inlineStr">
+        <is>
+          <t>Nilai Bulanan (Rp)</t>
+        </is>
+      </c>
+      <c r="F20" s="203" t="inlineStr">
+        <is>
+          <t>Keterangan Metrik Bisnis</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="204" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="205" t="inlineStr">
+        <is>
+          <t>Produksi PCO Jadi</t>
+        </is>
+      </c>
+      <c r="D21" s="204" t="inlineStr">
+        <is>
+          <t>520.000 kg (+- 520,00 ton)</t>
+        </is>
+      </c>
+      <c r="E21" s="215" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F21" s="216" t="inlineStr">
+        <is>
+          <t>26 hari kerja @ 20 Ton/hari produk jadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="204" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="205" t="inlineStr">
+        <is>
+          <t>Harga Jual Rata-Rata</t>
+        </is>
+      </c>
+      <c r="D22" s="204" t="inlineStr">
+        <is>
+          <t>Rp 8.300 / kg</t>
+        </is>
+      </c>
+      <c r="E22" s="209" t="n">
+        <v>4316000000</v>
+      </c>
+      <c r="F22" s="216" t="inlineStr">
+        <is>
+          <t>Harga jual off-taker B2B industri semen</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="204" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" s="217" t="inlineStr">
+        <is>
+          <t>OMZET PER BULAN</t>
+        </is>
+      </c>
+      <c r="D23" s="204" t="inlineStr">
+        <is>
+          <t>520.000 kg @ Rp 8.300</t>
+        </is>
+      </c>
+      <c r="E23" s="218">
+        <f>E22</f>
+        <v/>
+      </c>
+      <c r="F23" s="216" t="inlineStr">
+        <is>
+          <t>Penerimaan kotor penjualan bulanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="204" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" s="205" t="inlineStr">
+        <is>
+          <t>Biaya Produksi (Cash HPP)</t>
+        </is>
+      </c>
+      <c r="D24" s="204" t="inlineStr">
+        <is>
+          <t>Rp 4.487 / kg</t>
+        </is>
+      </c>
+      <c r="E24" s="209" t="n">
+        <v>2333240000</v>
+      </c>
+      <c r="F24" s="216" t="inlineStr">
+        <is>
+          <t>Raw Mat (Rp 2.000) + Pabrik (Rp 2.000) + Sewa Gudang (Rp 487)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="204" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" s="217" t="inlineStr">
+        <is>
+          <t>LABA KOTOR</t>
+        </is>
+      </c>
+      <c r="D25" s="204" t="inlineStr">
+        <is>
+          <t>Omzet - Cash HPP</t>
+        </is>
+      </c>
+      <c r="E25" s="219">
+        <f>E23-E24</f>
+        <v/>
+      </c>
+      <c r="F25" s="216" t="inlineStr">
+        <is>
+          <t>Laba kotor operasional sebelum biaya umum</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="204" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" s="205" t="inlineStr">
+        <is>
+          <t>Biaya Operasional Lain (utilitas, naker, legal, SG&amp;A)</t>
+        </is>
+      </c>
+      <c r="D26" s="204" t="inlineStr">
+        <is>
+          <t>Alokasi Pengelola</t>
+        </is>
+      </c>
+      <c r="E26" s="209" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="F26" s="216" t="inlineStr">
+        <is>
+          <t>Biaya operasional &amp; pemeliharaan berkala</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="204" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" s="217" t="inlineStr">
+        <is>
+          <t>EBITDA (PERKIRAAN)</t>
+        </is>
+      </c>
+      <c r="D27" s="204" t="inlineStr">
+        <is>
+          <t>Laba Kotor - Biaya Ops Lain</t>
+        </is>
+      </c>
+      <c r="E27" s="219">
+        <f>E25-E26</f>
+        <v/>
+      </c>
+      <c r="F27" s="216" t="inlineStr">
+        <is>
+          <t>Laba operasional sebelum beban depresiasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="204" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" s="205" t="inlineStr">
+        <is>
+          <t>Depresiasi Aset Mesin &amp; Gudang (5 Tahun)</t>
+        </is>
+      </c>
+      <c r="D28" s="204" t="inlineStr">
+        <is>
+          <t>Capex Rp 5 M / 60 Bulan</t>
+        </is>
+      </c>
+      <c r="E28" s="209" t="n">
+        <v>83200000</v>
+      </c>
+      <c r="F28" s="216" t="inlineStr">
+        <is>
+          <t>Rp 160 / kg (Pemulihan investasi Pihak Pertama)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="204" t="n">
+        <v>9</v>
+      </c>
+      <c r="C29" s="217" t="inlineStr">
+        <is>
+          <t>EAT (ESTIMASI LABA BERSIH BULANAN)</t>
+        </is>
+      </c>
+      <c r="D29" s="204" t="inlineStr">
+        <is>
+          <t>EBITDA - Depresiasi</t>
+        </is>
+      </c>
+      <c r="E29" s="220">
+        <f>E27-E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="216" t="inlineStr">
+        <is>
+          <t>Dasar pembagian hasil laba bersih (EAT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="201" t="inlineStr">
+        <is>
+          <t>5. PEMBAGIAN LABA BERSIH (EAT) 60% : 40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="202" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C32" s="203" t="inlineStr">
+        <is>
+          <t>Penerima Bagi Hasil</t>
+        </is>
+      </c>
+      <c r="D32" s="202" t="inlineStr">
+        <is>
+          <t>Porsi (%)</t>
+        </is>
+      </c>
+      <c r="E32" s="203" t="inlineStr">
+        <is>
+          <t>Bagi Hasil per Bulan (Rp)</t>
+        </is>
+      </c>
+      <c r="F32" s="203" t="inlineStr">
+        <is>
+          <t>Bagi Hasil per Tahun (Rp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="221" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="222" t="inlineStr">
+        <is>
+          <t>PIHAK PERTAMA: PT Pioner Nusantara Sukses (Pemodal)</t>
+        </is>
+      </c>
+      <c r="D33" s="206" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="E33" s="220">
+        <f>E29*0.6</f>
+        <v/>
+      </c>
+      <c r="F33" s="220">
+        <f>E33*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="221" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="222" t="inlineStr">
+        <is>
+          <t>PIHAK KEDUA: PT. Randu Agung Bersaudara (Pengelola)</t>
+        </is>
+      </c>
+      <c r="D34" s="207" t="inlineStr">
+        <is>
+          <t>40%</t>
+        </is>
+      </c>
+      <c r="E34" s="218">
+        <f>E29*0.4</f>
+        <v/>
+      </c>
+      <c r="F34" s="218">
+        <f>E34*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="223" t="inlineStr"/>
+      <c r="C35" s="224" t="inlineStr">
+        <is>
+          <t>TOTAL EAT TERDISTRIBUSI</t>
+        </is>
+      </c>
+      <c r="D35" s="225" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E35" s="226">
+        <f>E33+E34</f>
+        <v/>
+      </c>
+      <c r="F35" s="226">
+        <f>F33+F34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="208" t="inlineStr">
+        <is>
+          <t>6. INDIKATOR PENGEMBALIAN MODAL PEMODAL (PAYBACK PERIOD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="221" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="222" t="inlineStr">
+        <is>
+          <t>Total Investasi Capex Pihak Pertama</t>
+        </is>
+      </c>
+      <c r="D38" s="227" t="n"/>
+      <c r="E38" s="228">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="F38" s="229" t="inlineStr">
+        <is>
+          <t>Milik penuh Pihak Pertama</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="221" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" s="222" t="inlineStr">
+        <is>
+          <t>Penerimaan Laba Bulanan Pihak Pertama (60%)</t>
+        </is>
+      </c>
+      <c r="D39" s="227" t="n"/>
+      <c r="E39" s="228">
+        <f>E33</f>
+        <v/>
+      </c>
+      <c r="F39" s="229" t="inlineStr">
+        <is>
+          <t>Arus kas masuk bersih per bulan</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="221" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" s="230" t="inlineStr">
+        <is>
+          <t>Estimasi Payback Period (Bulan)</t>
+        </is>
+      </c>
+      <c r="D40" s="227" t="n"/>
+      <c r="E40" s="231">
+        <f>E38/E39</f>
+        <v/>
+      </c>
+      <c r="F40" s="229" t="inlineStr">
+        <is>
+          <t>Hanya butuh +- 4,42 Bulan untuk balik modal penuh!</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="221" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" s="230" t="inlineStr">
+        <is>
+          <t>Estimasi Payback Period (Tahun)</t>
+        </is>
+      </c>
+      <c r="D41" s="227" t="n"/>
+      <c r="E41" s="232">
+        <f>E40/12</f>
+        <v/>
+      </c>
+      <c r="F41" s="229" t="inlineStr">
+        <is>
+          <t>Sangat menarik (&lt; 0,5 Tahun)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="201" t="inlineStr">
+        <is>
+          <t>7. MATRIKS MANFAAT KERJASAMA BAGI KEDUA BELAH PIHAK</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="233" t="inlineStr">
+        <is>
+          <t>Pihak Pertama (Pemodal)</t>
+        </is>
+      </c>
+      <c r="E44" s="234" t="inlineStr">
+        <is>
+          <t>Pihak Kedua (Pengelola Operasional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="222" t="inlineStr">
+        <is>
+          <t>[v] Potensi return investasi sangat menarik (Payback +- 4,4 bulan)</t>
+        </is>
+      </c>
+      <c r="C45" s="235" t="n"/>
+      <c r="D45" s="235" t="n"/>
+      <c r="E45" s="222" t="inlineStr">
+        <is>
+          <t>[v] Mendapat bagian laba 40% dari EAT (Rp 753 jt/bln)</t>
+        </is>
+      </c>
+      <c r="F45" s="235" t="n"/>
+    </row>
+    <row r="46">
+      <c r="B46" s="222" t="inlineStr">
+        <is>
+          <t>[v] Aset mesin &amp; bangunan 100% tetap milik sah perusahaan</t>
+        </is>
+      </c>
+      <c r="C46" s="235" t="n"/>
+      <c r="D46" s="235" t="n"/>
+      <c r="E46" s="222" t="inlineStr">
+        <is>
+          <t>[v] Mengelola operasional secara penuh dan mandiri</t>
+        </is>
+      </c>
+      <c r="F46" s="235" t="n"/>
+    </row>
+    <row r="47">
+      <c r="B47" s="222" t="inlineStr">
+        <is>
+          <t>[v] Tidak perlu terlibat dalam operasional harian yang kompleks</t>
+        </is>
+      </c>
+      <c r="C47" s="235" t="n"/>
+      <c r="D47" s="235" t="n"/>
+      <c r="E47" s="222" t="inlineStr">
+        <is>
+          <t>[v] Mengembangkan pasar off-taker, perizinan, dan legalitas</t>
+        </is>
+      </c>
+      <c r="F47" s="235" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="222" t="inlineStr">
+        <is>
+          <t>[v] Ikut berkontribusi nyata pada energi bersih &amp; ekonomi sirkular</t>
+        </is>
+      </c>
+      <c r="C48" s="235" t="n"/>
+      <c r="D48" s="235" t="n"/>
+      <c r="E48" s="222" t="inlineStr">
+        <is>
+          <t>[v] Meningkatkan nilai dan reputasi perusahaan bersama</t>
+        </is>
+      </c>
+      <c r="F48" s="235" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B48:D48"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="B43:F43"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="B47:D47"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="E47:F47"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>